<commit_message>
[skip module] now NO CROP frame (for BIG model input)  after skip
</commit_message>
<xml_diff>
--- a/_TODO.xlsx
+++ b/_TODO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SyncData\paper2_main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C833ABB-2376-4490-AA56-7299F78F37BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CFCAD09-D519-4373-99CB-1011FF11FD49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17010" yWindow="285" windowWidth="28110" windowHeight="16035" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="62">
   <si>
     <t xml:space="preserve">Any articles, templates, or information provided by Smartsheet on the website are for reference only. While we strive to keep the information up to date and correct, we make no representations or warranties of any kind, express or implied, about the completeness, accuracy, reliability, suitability, or availability with respect to the website or the information, articles, templates, or related graphics contained on the website. Any reliance you place on such information is therefore strictly at your own risk. </t>
   </si>
@@ -1626,7 +1626,9 @@
       <c r="G12" s="39" t="s">
         <v>58</v>
       </c>
-      <c r="H12" s="41"/>
+      <c r="H12" s="41" t="s">
+        <v>37</v>
+      </c>
       <c r="I12" s="36"/>
       <c r="J12" s="36"/>
       <c r="K12" s="36"/>

</xml_diff>

<commit_message>
[opt_ranking udpate] update opt val selection results table using new ranking
</commit_message>
<xml_diff>
--- a/_TODO.xlsx
+++ b/_TODO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SyncData\paper2_main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F2DBC0B-5552-479E-9A51-F6BA8F944287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A994FE91-1BFE-4F71-B48C-125A95CE1CD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17010" yWindow="-120" windowWidth="28110" windowHeight="16440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1435,7 +1435,7 @@
         <v>60</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="E16" s="13" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
[update] fps now calc based on MainPC
</commit_message>
<xml_diff>
--- a/_TODO.xlsx
+++ b/_TODO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SyncData\paper2_main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{061675FC-93FA-45A4-B65E-5C09CC8A8663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{061D6398-94AF-4638-B560-97C8B06319C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17010" yWindow="-120" windowWidth="28110" windowHeight="16440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17010" yWindow="285" windowWidth="28110" windowHeight="16035" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Example Issue Tracking" sheetId="4" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="74">
   <si>
     <t>Status</t>
   </si>
@@ -273,6 +273,21 @@
   </si>
   <si>
     <t>On Hold</t>
+  </si>
+  <si>
+    <t>2026.04.21</t>
+  </si>
+  <si>
+    <t>iss18</t>
+  </si>
+  <si>
+    <t>update FPS of all table based on pre-computed NoTemp in MainPC</t>
+  </si>
+  <si>
+    <t>opt_accMotionDet</t>
+  </si>
+  <si>
+    <t>opt_Tpt</t>
   </si>
 </sst>
 </file>
@@ -1546,14 +1561,24 @@
     </row>
     <row r="20" spans="1:15" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A20" s="7"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
+      <c r="B20" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>8</v>
+      </c>
       <c r="F20" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="G20" s="16"/>
+      <c r="G20" s="16" t="s">
+        <v>71</v>
+      </c>
       <c r="H20" s="17"/>
       <c r="I20" s="7"/>
       <c r="J20" s="7"/>
@@ -6323,7 +6348,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7244F240-3E57-47A4-933B-A5E0C8789D48}">
-  <dimension ref="B2:H14"/>
+  <dimension ref="B2:H13"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="22.625" customWidth="1"/>
@@ -6386,7 +6411,7 @@
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>46</v>
@@ -6394,37 +6419,41 @@
       <c r="D4" s="2">
         <v>96</v>
       </c>
-      <c r="E4" s="2">
-        <v>275</v>
-      </c>
+      <c r="E4" s="2"/>
       <c r="F4" s="2" t="str">
-        <f>TEXT(E4/86400,"[h]:mm:ss")</f>
-        <v>0:04:35</v>
+        <f t="shared" ref="F4:F13" si="0">TEXT(E4/86400,"[h]:mm:ss")</f>
+        <v>0:00:00</v>
       </c>
       <c r="G4" s="2">
-        <f>D4*E4</f>
-        <v>26400</v>
+        <f t="shared" ref="G4:G13" si="1">D4*E4</f>
+        <v>0</v>
       </c>
       <c r="H4" s="2" t="str">
-        <f t="shared" ref="H4:H14" si="0">TEXT(G4/86400,"[h]:mm:ss")</f>
-        <v>7:20:00</v>
+        <f t="shared" ref="H4:H13" si="2">TEXT(G4/86400,"[h]:mm:ss")</f>
+        <v>0:00:00</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
+      <c r="B5" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="2">
+        <v>126</v>
+      </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2" t="str">
-        <f t="shared" ref="F5:F14" si="1">TEXT(E5/86400,"[h]:mm:ss")</f>
+        <f t="shared" si="0"/>
         <v>0:00:00</v>
       </c>
       <c r="G5" s="2">
-        <f t="shared" ref="G5:G14" si="2">D5*E5</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="H5" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0:00:00</v>
       </c>
     </row>
@@ -6434,15 +6463,15 @@
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0:00:00</v>
+      </c>
+      <c r="G6" s="2">
         <f t="shared" si="1"/>
-        <v>0:00:00</v>
-      </c>
-      <c r="G6" s="2">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2" t="str">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H6" s="2" t="str">
-        <f t="shared" si="0"/>
         <v>0:00:00</v>
       </c>
     </row>
@@ -6452,15 +6481,15 @@
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0:00:00</v>
+      </c>
+      <c r="G7" s="2">
         <f t="shared" si="1"/>
-        <v>0:00:00</v>
-      </c>
-      <c r="G7" s="2">
+        <v>0</v>
+      </c>
+      <c r="H7" s="2" t="str">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H7" s="2" t="str">
-        <f t="shared" si="0"/>
         <v>0:00:00</v>
       </c>
     </row>
@@ -6470,15 +6499,15 @@
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0:00:00</v>
+      </c>
+      <c r="G8" s="2">
         <f t="shared" si="1"/>
-        <v>0:00:00</v>
-      </c>
-      <c r="G8" s="2">
+        <v>0</v>
+      </c>
+      <c r="H8" s="2" t="str">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H8" s="2" t="str">
-        <f t="shared" si="0"/>
         <v>0:00:00</v>
       </c>
     </row>
@@ -6488,15 +6517,15 @@
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0:00:00</v>
+      </c>
+      <c r="G9" s="2">
         <f t="shared" si="1"/>
-        <v>0:00:00</v>
-      </c>
-      <c r="G9" s="2">
+        <v>0</v>
+      </c>
+      <c r="H9" s="2" t="str">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H9" s="2" t="str">
-        <f t="shared" si="0"/>
         <v>0:00:00</v>
       </c>
     </row>
@@ -6506,15 +6535,15 @@
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0:00:00</v>
+      </c>
+      <c r="G10" s="2">
         <f t="shared" si="1"/>
-        <v>0:00:00</v>
-      </c>
-      <c r="G10" s="2">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2" t="str">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H10" s="2" t="str">
-        <f t="shared" si="0"/>
         <v>0:00:00</v>
       </c>
     </row>
@@ -6524,15 +6553,15 @@
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0:00:00</v>
+      </c>
+      <c r="G11" s="2">
         <f t="shared" si="1"/>
-        <v>0:00:00</v>
-      </c>
-      <c r="G11" s="2">
+        <v>0</v>
+      </c>
+      <c r="H11" s="2" t="str">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H11" s="2" t="str">
-        <f t="shared" si="0"/>
         <v>0:00:00</v>
       </c>
     </row>
@@ -6542,15 +6571,15 @@
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>0:00:00</v>
+      </c>
+      <c r="G12" s="2">
         <f t="shared" si="1"/>
-        <v>0:00:00</v>
-      </c>
-      <c r="G12" s="2">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2" t="str">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H12" s="2" t="str">
-        <f t="shared" si="0"/>
         <v>0:00:00</v>
       </c>
     </row>
@@ -6560,33 +6589,15 @@
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>0:00:00</v>
-      </c>
-      <c r="G13" s="2">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H13" s="2" t="str">
         <f t="shared" si="0"/>
         <v>0:00:00</v>
       </c>
-    </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2" t="str">
+      <c r="G13" s="2">
         <f t="shared" si="1"/>
-        <v>0:00:00</v>
-      </c>
-      <c r="G14" s="2">
+        <v>0</v>
+      </c>
+      <c r="H13" s="2" t="str">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H14" s="2" t="str">
-        <f t="shared" si="0"/>
         <v>0:00:00</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update big model training info
</commit_message>
<xml_diff>
--- a/_TODO.xlsx
+++ b/_TODO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SyncData\paper2_main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{061D6398-94AF-4638-B560-97C8B06319C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41F43721-C253-4D39-992A-C161B453F957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17010" yWindow="285" windowWidth="28110" windowHeight="16035" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17010" yWindow="-120" windowWidth="28110" windowHeight="16440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Example Issue Tracking" sheetId="4" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="87">
   <si>
     <t>Status</t>
   </si>
@@ -263,9 +263,6 @@
     <t>iss16</t>
   </si>
   <si>
-    <t>Skip  module with feedback from BIG MODEL (if big model confirm fire/smoke fore few frames, then ignore SKIP for a specific period)</t>
-  </si>
-  <si>
     <t>iss17</t>
   </si>
   <si>
@@ -288,6 +285,48 @@
   </si>
   <si>
     <t>opt_Tpt</t>
+  </si>
+  <si>
+    <t>Eager mode: implementation + update report (Hyperparam search on Val + Results on Test set)</t>
+  </si>
+  <si>
+    <t>2026.05.12</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Update the text describing the training of BIG Model</t>
+  </si>
+  <si>
+    <t>iss19</t>
+  </si>
+  <si>
+    <t>RE-check + Update all Paper2 content (to make sure it consistent)</t>
+  </si>
+  <si>
+    <t>iss20</t>
+  </si>
+  <si>
+    <t>Merge Paper2 Content into Thesis</t>
+  </si>
+  <si>
+    <t>iss21</t>
+  </si>
+  <si>
+    <t>Revise Chapter 1 (Intro) + Chap2 (Literature) + Chap5 (Conclusion + Future) in the Thesis</t>
+  </si>
+  <si>
+    <t>iss22</t>
+  </si>
+  <si>
+    <t>iss23</t>
+  </si>
+  <si>
+    <t>Prepare slides for Thesis Defense</t>
+  </si>
+  <si>
+    <t>Final review the Thesis before sending out for Committee 's Review</t>
   </si>
 </sst>
 </file>
@@ -481,7 +520,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -547,6 +586,10 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1463,7 +1506,9 @@
       <c r="G16" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="H16" s="17"/>
+      <c r="H16" s="17" t="s">
+        <v>19</v>
+      </c>
       <c r="I16" s="7"/>
       <c r="J16" s="7"/>
       <c r="K16" s="7"/>
@@ -1475,22 +1520,22 @@
     <row r="17" spans="1:15" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A17" s="7"/>
       <c r="B17" s="12" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>68</v>
+        <v>6</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F17" s="13" t="s">
         <v>9</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="H17" s="17"/>
       <c r="I17" s="7"/>
@@ -1501,27 +1546,29 @@
       <c r="N17" s="7"/>
       <c r="O17" s="7"/>
     </row>
-    <row r="18" spans="1:15" s="11" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A18" s="7"/>
       <c r="B18" s="12" t="s">
         <v>54</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F18" s="13" t="s">
         <v>9</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="H18" s="17"/>
+        <v>63</v>
+      </c>
+      <c r="H18" s="17" t="s">
+        <v>19</v>
+      </c>
       <c r="I18" s="7"/>
       <c r="J18" s="7"/>
       <c r="K18" s="7"/>
@@ -1536,10 +1583,10 @@
         <v>54</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E19" s="13" t="s">
         <v>8</v>
@@ -1548,7 +1595,7 @@
         <v>9</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H19" s="17"/>
       <c r="I19" s="7"/>
@@ -1562,10 +1609,10 @@
     <row r="20" spans="1:15" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A20" s="7"/>
       <c r="B20" s="12" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="D20" s="13" t="s">
         <v>56</v>
@@ -1574,10 +1621,10 @@
         <v>8</v>
       </c>
       <c r="F20" s="13" t="s">
-        <v>9</v>
+        <v>75</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H20" s="17"/>
       <c r="I20" s="7"/>
@@ -1590,14 +1637,24 @@
     </row>
     <row r="21" spans="1:15" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A21" s="7"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
+      <c r="B21" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>8</v>
+      </c>
       <c r="F21" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="G21" s="16"/>
+        <v>75</v>
+      </c>
+      <c r="G21" s="16" t="s">
+        <v>76</v>
+      </c>
       <c r="H21" s="17"/>
       <c r="I21" s="7"/>
       <c r="J21" s="7"/>
@@ -1609,14 +1666,24 @@
     </row>
     <row r="22" spans="1:15" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A22" s="7"/>
-      <c r="B22" s="12"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
+      <c r="B22" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>8</v>
+      </c>
       <c r="F22" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="G22" s="16"/>
+        <v>75</v>
+      </c>
+      <c r="G22" s="21" t="s">
+        <v>78</v>
+      </c>
       <c r="H22" s="17"/>
       <c r="I22" s="7"/>
       <c r="J22" s="7"/>
@@ -1628,14 +1695,24 @@
     </row>
     <row r="23" spans="1:15" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A23" s="7"/>
-      <c r="B23" s="12"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
+      <c r="B23" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>8</v>
+      </c>
       <c r="F23" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="G23" s="16"/>
+        <v>75</v>
+      </c>
+      <c r="G23" s="16" t="s">
+        <v>80</v>
+      </c>
       <c r="H23" s="17"/>
       <c r="I23" s="7"/>
       <c r="J23" s="7"/>
@@ -1647,14 +1724,24 @@
     </row>
     <row r="24" spans="1:15" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A24" s="7"/>
-      <c r="B24" s="12"/>
-      <c r="C24" s="12"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
+      <c r="B24" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>8</v>
+      </c>
       <c r="F24" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="G24" s="16"/>
+        <v>10</v>
+      </c>
+      <c r="G24" s="16" t="s">
+        <v>82</v>
+      </c>
       <c r="H24" s="17"/>
       <c r="I24" s="7"/>
       <c r="J24" s="7"/>
@@ -1666,14 +1753,24 @@
     </row>
     <row r="25" spans="1:15" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A25" s="7"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
+      <c r="B25" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>8</v>
+      </c>
       <c r="F25" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="G25" s="16"/>
+        <v>10</v>
+      </c>
+      <c r="G25" s="21" t="s">
+        <v>86</v>
+      </c>
       <c r="H25" s="17"/>
       <c r="I25" s="7"/>
       <c r="J25" s="7"/>
@@ -1685,14 +1782,24 @@
     </row>
     <row r="26" spans="1:15" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="7"/>
-      <c r="B26" s="12"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
+      <c r="B26" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>8</v>
+      </c>
       <c r="F26" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="G26" s="16"/>
+      <c r="G26" s="16" t="s">
+        <v>85</v>
+      </c>
       <c r="H26" s="17"/>
       <c r="I26" s="7"/>
       <c r="J26" s="7"/>
@@ -6290,6 +6397,10 @@
       <c r="H709" s="20"/>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:H20">
+    <sortCondition ref="D3:D20"/>
+    <sortCondition ref="B3:B20"/>
+  </sortState>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="D3:F26">
     <cfRule type="containsText" dxfId="10" priority="9" operator="containsText" text="Closed">
@@ -6332,7 +6443,7 @@
   </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F3:F26" xr:uid="{0FE1C215-D2BB-457C-B71B-3AD1725D56C1}">
-      <formula1>#REF!</formula1>
+      <formula1>"Critical, High, Medium, Low"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:D26" xr:uid="{49DD096F-692D-432E-8379-3E1D921F826C}">
       <formula1>"Open, Closed, On Hold"</formula1>
@@ -6411,7 +6522,7 @@
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>46</v>
@@ -6435,7 +6546,7 @@
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>46</v>

</xml_diff>